<commit_message>
SHD sanity suite getting flight numbers - 17-11-2025
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/FlightNumbers.xlsx
+++ b/src/test/java/TestData/FlightNumbers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Harshitha Rajesh\Copa_SHD_API_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2121E83-3AA8-4DD4-962B-E673DE864B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F72C762-C19F-4447-A216-7C327A8103BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
   <si>
     <t>Route</t>
   </si>
@@ -100,86 +100,197 @@
     <t>PTY-MIA</t>
   </si>
   <si>
+    <t>419</t>
+  </si>
+  <si>
+    <t>334</t>
+  </si>
+  <si>
+    <t>485</t>
+  </si>
+  <si>
+    <t>240</t>
+  </si>
+  <si>
+    <t>427</t>
+  </si>
+  <si>
+    <t>441</t>
+  </si>
+  <si>
+    <t>Flight 7</t>
+  </si>
+  <si>
+    <t>PTY-ORD</t>
+  </si>
+  <si>
+    <t>228</t>
+  </si>
+  <si>
+    <t>235</t>
+  </si>
+  <si>
+    <t>PTY-GYE</t>
+  </si>
+  <si>
+    <t>273</t>
+  </si>
+  <si>
+    <t>258</t>
+  </si>
+  <si>
+    <t>378</t>
+  </si>
+  <si>
+    <t>213</t>
+  </si>
+  <si>
+    <t>301</t>
+  </si>
+  <si>
+    <t>311</t>
+  </si>
+  <si>
+    <t>GYE-PTY</t>
+  </si>
+  <si>
+    <t>214</t>
+  </si>
+  <si>
+    <t>313</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
+    <t>377</t>
+  </si>
+  <si>
+    <t>272</t>
+  </si>
+  <si>
+    <t>379</t>
+  </si>
+  <si>
     <t>226</t>
   </si>
   <si>
-    <t>419</t>
-  </si>
-  <si>
-    <t>334</t>
-  </si>
-  <si>
-    <t>485</t>
-  </si>
-  <si>
-    <t>240</t>
-  </si>
-  <si>
-    <t>427</t>
-  </si>
-  <si>
-    <t>441</t>
-  </si>
-  <si>
-    <t>Flight 7</t>
-  </si>
-  <si>
-    <t>PTY-ORD</t>
-  </si>
-  <si>
-    <t>228</t>
-  </si>
-  <si>
-    <t>235</t>
-  </si>
-  <si>
-    <t>PTY-GYE</t>
-  </si>
-  <si>
-    <t>273</t>
-  </si>
-  <si>
-    <t>258</t>
-  </si>
-  <si>
-    <t>378</t>
-  </si>
-  <si>
-    <t>213</t>
-  </si>
-  <si>
-    <t>301</t>
-  </si>
-  <si>
-    <t>311</t>
-  </si>
-  <si>
-    <t>GYE-PTY</t>
-  </si>
-  <si>
-    <t>214</t>
-  </si>
-  <si>
-    <t>313</t>
-  </si>
-  <si>
-    <t>300</t>
-  </si>
-  <si>
-    <t>377</t>
-  </si>
-  <si>
-    <t>272</t>
-  </si>
-  <si>
-    <t>379</t>
+    <t>BOG-PTY</t>
+  </si>
+  <si>
+    <t>PTY-BOG</t>
+  </si>
+  <si>
+    <t>MCO-PTY</t>
+  </si>
+  <si>
+    <t>PTY-MCO</t>
+  </si>
+  <si>
+    <t>MIA-PTY</t>
+  </si>
+  <si>
+    <t>837</t>
+  </si>
+  <si>
+    <t>495</t>
+  </si>
+  <si>
+    <t>431</t>
+  </si>
+  <si>
+    <t>412</t>
+  </si>
+  <si>
+    <t>416</t>
+  </si>
+  <si>
+    <t>335</t>
+  </si>
+  <si>
+    <t>244</t>
+  </si>
+  <si>
+    <t>243</t>
+  </si>
+  <si>
+    <t>274</t>
+  </si>
+  <si>
+    <t>332</t>
+  </si>
+  <si>
+    <t>413</t>
+  </si>
+  <si>
+    <t>415</t>
+  </si>
+  <si>
+    <t>411</t>
+  </si>
+  <si>
+    <t>494</t>
+  </si>
+  <si>
+    <t>446</t>
+  </si>
+  <si>
+    <t>862</t>
+  </si>
+  <si>
+    <t>867</t>
+  </si>
+  <si>
+    <t>478</t>
+  </si>
+  <si>
+    <t>434</t>
+  </si>
+  <si>
+    <t>285</t>
+  </si>
+  <si>
+    <t>435</t>
+  </si>
+  <si>
+    <t>239</t>
+  </si>
+  <si>
+    <t>479</t>
+  </si>
+  <si>
+    <t>868</t>
+  </si>
+  <si>
+    <t>459</t>
+  </si>
+  <si>
+    <t>445</t>
+  </si>
+  <si>
+    <t>246</t>
+  </si>
+  <si>
+    <t>433</t>
+  </si>
+  <si>
+    <t>440</t>
+  </si>
+  <si>
+    <t>481</t>
+  </si>
+  <si>
+    <t>333</t>
+  </si>
+  <si>
+    <t>227</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -187,16 +298,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -204,13 +329,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -545,7 +687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
@@ -553,173 +695,310 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="B6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="B7" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="G8" t="s">
-        <v>50</v>
-      </c>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H13" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Arindam's and Harshitha's changes pushed - 12-12-2025
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/FlightNumbers.xlsx
+++ b/src/test/java/TestData/FlightNumbers.xlsx
@@ -1,26 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29607"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Harshitha Rajesh\Copa_SHD_API_WebServices\src\test\java\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation\Copa_API_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F72C762-C19F-4447-A216-7C327A8103BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{32F8D27F-933E-40FF-AEA7-B998BB66F101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE30DF59-32FD-43C5-B6F3-86BCF443DB68}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Flight Data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="132">
   <si>
     <t>Route</t>
   </si>
@@ -28,6 +44,24 @@
     <t>Flight 1</t>
   </si>
   <si>
+    <t>Flight 2</t>
+  </si>
+  <si>
+    <t>Flight 3</t>
+  </si>
+  <si>
+    <t>Flight 4</t>
+  </si>
+  <si>
+    <t>Flight 5</t>
+  </si>
+  <si>
+    <t>Flight 6</t>
+  </si>
+  <si>
+    <t>Flight 7</t>
+  </si>
+  <si>
     <t>PTY-CUN</t>
   </si>
   <si>
@@ -37,33 +71,18 @@
     <t>122</t>
   </si>
   <si>
-    <t>Flight 2</t>
-  </si>
-  <si>
     <t>316</t>
   </si>
   <si>
-    <t>Flight 3</t>
-  </si>
-  <si>
     <t>113</t>
   </si>
   <si>
-    <t>Flight 4</t>
-  </si>
-  <si>
     <t>324</t>
   </si>
   <si>
-    <t>Flight 5</t>
-  </si>
-  <si>
     <t>103</t>
   </si>
   <si>
-    <t>Flight 6</t>
-  </si>
-  <si>
     <t>PTY-MEX</t>
   </si>
   <si>
@@ -100,6 +119,9 @@
     <t>PTY-MIA</t>
   </si>
   <si>
+    <t>226</t>
+  </si>
+  <si>
     <t>419</t>
   </si>
   <si>
@@ -118,9 +140,6 @@
     <t>441</t>
   </si>
   <si>
-    <t>Flight 7</t>
-  </si>
-  <si>
     <t>PTY-ORD</t>
   </si>
   <si>
@@ -133,15 +152,15 @@
     <t>PTY-GYE</t>
   </si>
   <si>
+    <t>258</t>
+  </si>
+  <si>
+    <t>378</t>
+  </si>
+  <si>
     <t>273</t>
   </si>
   <si>
-    <t>258</t>
-  </si>
-  <si>
-    <t>378</t>
-  </si>
-  <si>
     <t>213</t>
   </si>
   <si>
@@ -172,102 +191,99 @@
     <t>379</t>
   </si>
   <si>
-    <t>226</t>
-  </si>
-  <si>
     <t>BOG-PTY</t>
   </si>
   <si>
+    <t>837</t>
+  </si>
+  <si>
+    <t>495</t>
+  </si>
+  <si>
+    <t>431</t>
+  </si>
+  <si>
+    <t>412</t>
+  </si>
+  <si>
+    <t>416</t>
+  </si>
+  <si>
+    <t>335</t>
+  </si>
+  <si>
+    <t>244</t>
+  </si>
+  <si>
     <t>PTY-BOG</t>
   </si>
   <si>
+    <t>243</t>
+  </si>
+  <si>
+    <t>274</t>
+  </si>
+  <si>
+    <t>332</t>
+  </si>
+  <si>
+    <t>413</t>
+  </si>
+  <si>
+    <t>415</t>
+  </si>
+  <si>
+    <t>411</t>
+  </si>
+  <si>
+    <t>494</t>
+  </si>
+  <si>
     <t>MCO-PTY</t>
   </si>
   <si>
+    <t>435</t>
+  </si>
+  <si>
+    <t>239</t>
+  </si>
+  <si>
+    <t>479</t>
+  </si>
+  <si>
+    <t>868</t>
+  </si>
+  <si>
+    <t>459</t>
+  </si>
+  <si>
+    <t>445</t>
+  </si>
+  <si>
     <t>PTY-MCO</t>
   </si>
   <si>
+    <t>446</t>
+  </si>
+  <si>
+    <t>862</t>
+  </si>
+  <si>
+    <t>867</t>
+  </si>
+  <si>
+    <t>478</t>
+  </si>
+  <si>
+    <t>434</t>
+  </si>
+  <si>
+    <t>285</t>
+  </si>
+  <si>
     <t>MIA-PTY</t>
   </si>
   <si>
-    <t>837</t>
-  </si>
-  <si>
-    <t>495</t>
-  </si>
-  <si>
-    <t>431</t>
-  </si>
-  <si>
-    <t>412</t>
-  </si>
-  <si>
-    <t>416</t>
-  </si>
-  <si>
-    <t>335</t>
-  </si>
-  <si>
-    <t>244</t>
-  </si>
-  <si>
-    <t>243</t>
-  </si>
-  <si>
-    <t>274</t>
-  </si>
-  <si>
-    <t>332</t>
-  </si>
-  <si>
-    <t>413</t>
-  </si>
-  <si>
-    <t>415</t>
-  </si>
-  <si>
-    <t>411</t>
-  </si>
-  <si>
-    <t>494</t>
-  </si>
-  <si>
-    <t>446</t>
-  </si>
-  <si>
-    <t>862</t>
-  </si>
-  <si>
-    <t>867</t>
-  </si>
-  <si>
-    <t>478</t>
-  </si>
-  <si>
-    <t>434</t>
-  </si>
-  <si>
-    <t>285</t>
-  </si>
-  <si>
-    <t>435</t>
-  </si>
-  <si>
-    <t>239</t>
-  </si>
-  <si>
-    <t>479</t>
-  </si>
-  <si>
-    <t>868</t>
-  </si>
-  <si>
-    <t>459</t>
-  </si>
-  <si>
-    <t>445</t>
-  </si>
-  <si>
     <t>246</t>
   </si>
   <si>
@@ -284,13 +300,145 @@
   </si>
   <si>
     <t>227</t>
+  </si>
+  <si>
+    <t>PTY-EZE</t>
+  </si>
+  <si>
+    <t>219</t>
+  </si>
+  <si>
+    <t>329</t>
+  </si>
+  <si>
+    <t>346</t>
+  </si>
+  <si>
+    <t>454</t>
+  </si>
+  <si>
+    <t>367</t>
+  </si>
+  <si>
+    <t>PTY-SAL</t>
+  </si>
+  <si>
+    <t>816</t>
+  </si>
+  <si>
+    <t>881</t>
+  </si>
+  <si>
+    <t>878</t>
+  </si>
+  <si>
+    <t>PTY-LIM</t>
+  </si>
+  <si>
+    <t>761</t>
+  </si>
+  <si>
+    <t>493</t>
+  </si>
+  <si>
+    <t>489</t>
+  </si>
+  <si>
+    <t>838</t>
+  </si>
+  <si>
+    <t>PTY-SDQ</t>
+  </si>
+  <si>
+    <t>463</t>
+  </si>
+  <si>
+    <t>298</t>
+  </si>
+  <si>
+    <t>268</t>
+  </si>
+  <si>
+    <t>PTY-GRU</t>
+  </si>
+  <si>
+    <t>701</t>
+  </si>
+  <si>
+    <t>725</t>
+  </si>
+  <si>
+    <t>800</t>
+  </si>
+  <si>
+    <t>743</t>
+  </si>
+  <si>
+    <t>759</t>
+  </si>
+  <si>
+    <t>COR-PTY</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>LAX-IAH</t>
+  </si>
+  <si>
+    <t>644</t>
+  </si>
+  <si>
+    <t>GRU-PTY</t>
+  </si>
+  <si>
+    <t>702</t>
+  </si>
+  <si>
+    <t>758</t>
+  </si>
+  <si>
+    <t>841</t>
+  </si>
+  <si>
+    <t>744</t>
+  </si>
+  <si>
+    <t>700</t>
+  </si>
+  <si>
+    <t> </t>
+  </si>
+  <si>
+    <t>GUA-PTY</t>
+  </si>
+  <si>
+    <t>361</t>
+  </si>
+  <si>
+    <t>384</t>
+  </si>
+  <si>
+    <t>407</t>
+  </si>
+  <si>
+    <t>389</t>
+  </si>
+  <si>
+    <t>PTY-SFO</t>
+  </si>
+  <si>
+    <t>382</t>
+  </si>
+  <si>
+    <t>601</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -305,6 +453,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -321,7 +475,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -344,15 +498,42 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -687,14 +868,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="8" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="8" width="7.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -702,125 +883,125 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="C2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="E2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -828,157 +1009,157 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>39</v>
       </c>
+      <c r="D7" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="E7" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8">
       <c r="A8" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8">
       <c r="A9" s="2" t="s">
         <v>51</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="3" t="s">
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="B10" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="H10" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="F10" s="3" t="s">
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="B11" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B11" s="3" t="s">
+      <c r="D11" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E12" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>82</v>
@@ -999,6 +1180,212 @@
         <v>87</v>
       </c>
       <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G14" s="3"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G18" s="3"/>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+    </row>
+    <row r="21" spans="1:8" ht="15">
+      <c r="A21" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="15">
+      <c r="A22" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="15">
+      <c r="A23" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>123</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Code changes for Mahalakshmi on 16/02/2026
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/FlightNumbers.xlsx
+++ b/src/test/java/TestData/FlightNumbers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29607"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation\Copa_API_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{32F8D27F-933E-40FF-AEA7-B998BB66F101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE30DF59-32FD-43C5-B6F3-86BCF443DB68}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72616EB8-692E-44BE-8326-5E6D6C298657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="90" yWindow="460" windowWidth="19180" windowHeight="10080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Flight Data" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="181">
   <si>
     <t>Route</t>
   </si>
@@ -416,7 +416,7 @@
     <t>361</t>
   </si>
   <si>
-    <t>384</t>
+    <t>183</t>
   </si>
   <si>
     <t>407</t>
@@ -432,13 +432,160 @@
   </si>
   <si>
     <t>601</t>
+  </si>
+  <si>
+    <t>PTY-IAH</t>
+  </si>
+  <si>
+    <t>1927</t>
+  </si>
+  <si>
+    <t>1933</t>
+  </si>
+  <si>
+    <t>1249</t>
+  </si>
+  <si>
+    <t>1031</t>
+  </si>
+  <si>
+    <t>LAX-PTY</t>
+  </si>
+  <si>
+    <t>306</t>
+  </si>
+  <si>
+    <t>473</t>
+  </si>
+  <si>
+    <t>362</t>
+  </si>
+  <si>
+    <t>SAL-PTY</t>
+  </si>
+  <si>
+    <t>879</t>
+  </si>
+  <si>
+    <t>884</t>
+  </si>
+  <si>
+    <t>871</t>
+  </si>
+  <si>
+    <t>PTY-SCL</t>
+  </si>
+  <si>
+    <t>395</t>
+  </si>
+  <si>
+    <t>497</t>
+  </si>
+  <si>
+    <t>171</t>
+  </si>
+  <si>
+    <t>474</t>
+  </si>
+  <si>
+    <t>277</t>
+  </si>
+  <si>
+    <t>SCL-PTY</t>
+  </si>
+  <si>
+    <t>475</t>
+  </si>
+  <si>
+    <t>276</t>
+  </si>
+  <si>
+    <t>396</t>
+  </si>
+  <si>
+    <t>498</t>
+  </si>
+  <si>
+    <t>174</t>
+  </si>
+  <si>
+    <t>118</t>
+  </si>
+  <si>
+    <t>MEX-PTY</t>
+  </si>
+  <si>
+    <t>195</t>
+  </si>
+  <si>
+    <t>137</t>
+  </si>
+  <si>
+    <t>121</t>
+  </si>
+  <si>
+    <t>PTY-GUA</t>
+  </si>
+  <si>
+    <t>391</t>
+  </si>
+  <si>
+    <t>380</t>
+  </si>
+  <si>
+    <t>358</t>
+  </si>
+  <si>
+    <t>390</t>
+  </si>
+  <si>
+    <t>LIM-PTY</t>
+  </si>
+  <si>
+    <t>PTY-SJO</t>
+  </si>
+  <si>
+    <t>338</t>
+  </si>
+  <si>
+    <t>264</t>
+  </si>
+  <si>
+    <t>462</t>
+  </si>
+  <si>
+    <t>787</t>
+  </si>
+  <si>
+    <t>818</t>
+  </si>
+  <si>
+    <t>460</t>
+  </si>
+  <si>
+    <t>192</t>
+  </si>
+  <si>
+    <t>135</t>
+  </si>
+  <si>
+    <t>401</t>
+  </si>
+  <si>
+    <t>IAH-PTY</t>
+  </si>
+  <si>
+    <t>1932</t>
+  </si>
+  <si>
+    <t>1934</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -460,6 +607,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -475,7 +628,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -522,18 +675,128 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -868,14 +1131,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H23"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:H34"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="8" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="8" width="7.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -901,7 +1164,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -925,7 +1188,7 @@
       </c>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -949,7 +1212,7 @@
       </c>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
@@ -962,12 +1225,14 @@
       <c r="D4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="2"/>
+      <c r="E4" s="3" t="s">
+        <v>177</v>
+      </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>26</v>
       </c>
@@ -993,7 +1258,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>34</v>
       </c>
@@ -1009,7 +1274,7 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>37</v>
       </c>
@@ -1033,7 +1298,7 @@
       </c>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>44</v>
       </c>
@@ -1057,7 +1322,7 @@
       </c>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>51</v>
       </c>
@@ -1083,7 +1348,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>59</v>
       </c>
@@ -1109,7 +1374,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>67</v>
       </c>
@@ -1133,7 +1398,7 @@
       </c>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>74</v>
       </c>
@@ -1157,7 +1422,7 @@
       </c>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>81</v>
       </c>
@@ -1181,7 +1446,7 @@
       </c>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>88</v>
       </c>
@@ -1203,7 +1468,7 @@
       <c r="G14" s="3"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>94</v>
       </c>
@@ -1221,7 +1486,7 @@
       <c r="G15" s="3"/>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>98</v>
       </c>
@@ -1241,7 +1506,7 @@
       <c r="G16" s="3"/>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>103</v>
       </c>
@@ -1259,7 +1524,7 @@
       <c r="G17" s="3"/>
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>107</v>
       </c>
@@ -1281,7 +1546,7 @@
       <c r="G18" s="3"/>
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>113</v>
       </c>
@@ -1295,7 +1560,7 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>115</v>
       </c>
@@ -1309,7 +1574,7 @@
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
-    <row r="21" spans="1:8" ht="15">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>117</v>
       </c>
@@ -1335,7 +1600,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
         <v>124</v>
       </c>
@@ -1361,7 +1626,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
         <v>129</v>
       </c>
@@ -1387,7 +1652,278 @@
         <v>123</v>
       </c>
     </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A24" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="E24" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A25" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="D25" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="D26" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="G26" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="H26" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="E27" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="H27" s="12" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A28" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="C28" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="D28" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="E28" s="18" t="s">
+        <v>155</v>
+      </c>
+      <c r="F28" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="G28" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="H28" s="14" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A29" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="H29" s="8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A30" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="H30" s="8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A31" s="19" t="s">
+        <v>167</v>
+      </c>
+      <c r="B31" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="C31" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="E31" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="F31" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="G31" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="H31" s="20" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A32" s="21" t="s">
+        <v>168</v>
+      </c>
+      <c r="B32" s="24" t="s">
+        <v>172</v>
+      </c>
+      <c r="C32" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="D32" s="24" t="s">
+        <v>174</v>
+      </c>
+      <c r="E32" s="24" t="s">
+        <v>175</v>
+      </c>
+      <c r="F32" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="G32" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="H32" s="22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A33" s="25" t="s">
+        <v>158</v>
+      </c>
+      <c r="B33" s="26" t="s">
+        <v>160</v>
+      </c>
+      <c r="C33" s="26" t="s">
+        <v>161</v>
+      </c>
+      <c r="D33" s="26" t="s">
+        <v>176</v>
+      </c>
+      <c r="E33" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A34" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B34" s="27" t="s">
+        <v>179</v>
+      </c>
+      <c r="C34" s="27" t="s">
+        <v>180</v>
+      </c>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+    </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Arindam faker code changes on 17/04/2026
</commit_message>
<xml_diff>
--- a/src/test/java/TestData/FlightNumbers.xlsx
+++ b/src/test/java/TestData/FlightNumbers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation\Copa_API_WebServices\src\test\java\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72616EB8-692E-44BE-8326-5E6D6C298657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F0EA771-3E6C-418A-A07C-E7C3F8A93CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="90" yWindow="460" windowWidth="19180" windowHeight="10080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="0" windowWidth="19180" windowHeight="10080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Flight Data" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="182">
   <si>
     <t>Route</t>
   </si>
@@ -579,6 +579,9 @@
   </si>
   <si>
     <t>1934</t>
+  </si>
+  <si>
+    <t>001</t>
   </si>
 </sst>
 </file>
@@ -1683,16 +1686,16 @@
         <v>137</v>
       </c>
       <c r="B25" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="C25" s="16" t="s">
         <v>138</v>
       </c>
-      <c r="C25" s="16" t="s">
+      <c r="D25" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="D25" s="16" t="s">
+      <c r="E25" s="16" t="s">
         <v>140</v>
-      </c>
-      <c r="E25" s="10" t="s">
-        <v>123</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>123</v>

</xml_diff>